<commit_message>
cambios excel y json
</commit_message>
<xml_diff>
--- a/data/INVENTARIO 2026 MILLER.xlsx
+++ b/data/INVENTARIO 2026 MILLER.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlos.garcia\Desktop\github\inventario_eic\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlos.garcia\Downloads\INVENTARIOS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC13BEEB-3685-4681-883C-2638725FCAFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{901FD746-B77D-4EAC-BEDE-B70BF07F2CEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{5D49649A-3F74-4AF5-B76C-DA0070D63EDA}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1999" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2052" uniqueCount="133">
   <si>
     <t>NUMERO DE INVENTARIO</t>
   </si>
@@ -427,12 +427,24 @@
   <si>
     <t>BUTACO BUTACO DROP ESTRUCTURA METALICA ACABADO ELECTROSTATICO,  PROTECCION UV. ALTURA 63CM</t>
   </si>
+  <si>
+    <t>GEOMATICA</t>
+  </si>
+  <si>
+    <t>OFICINA JHON CACERES</t>
+  </si>
+  <si>
+    <t>ABP 106</t>
+  </si>
+  <si>
+    <t>ABP 107</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -444,6 +456,12 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -5322,7 +5340,9 @@
       <c r="B224" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="C224" s="3"/>
+      <c r="C224" s="3" t="s">
+        <v>129</v>
+      </c>
       <c r="D224" s="3"/>
       <c r="E224" s="3" t="s">
         <v>6</v>
@@ -5342,7 +5362,9 @@
       <c r="B225" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="C225" s="3"/>
+      <c r="C225" s="3" t="s">
+        <v>129</v>
+      </c>
       <c r="D225" s="3"/>
       <c r="E225" s="3" t="s">
         <v>6</v>
@@ -5782,7 +5804,9 @@
       <c r="B247" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C247" s="3"/>
+      <c r="C247" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="D247" s="3"/>
       <c r="E247" s="3" t="s">
         <v>6</v>
@@ -5802,7 +5826,9 @@
       <c r="B248" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C248" s="3"/>
+      <c r="C248" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="D248" s="3"/>
       <c r="E248" s="3" t="s">
         <v>6</v>
@@ -5822,7 +5848,9 @@
       <c r="B249" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C249" s="3"/>
+      <c r="C249" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="D249" s="3"/>
       <c r="E249" s="3" t="s">
         <v>6</v>
@@ -5842,7 +5870,9 @@
       <c r="B250" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C250" s="3"/>
+      <c r="C250" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="D250" s="3"/>
       <c r="E250" s="3" t="s">
         <v>6</v>
@@ -5862,7 +5892,9 @@
       <c r="B251" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C251" s="3"/>
+      <c r="C251" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="D251" s="3"/>
       <c r="E251" s="3" t="s">
         <v>6</v>
@@ -5882,7 +5914,9 @@
       <c r="B252" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C252" s="3"/>
+      <c r="C252" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="D252" s="3"/>
       <c r="E252" s="3" t="s">
         <v>6</v>
@@ -5902,7 +5936,9 @@
       <c r="B253" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C253" s="3"/>
+      <c r="C253" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="D253" s="3"/>
       <c r="E253" s="3" t="s">
         <v>6</v>
@@ -5922,7 +5958,9 @@
       <c r="B254" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C254" s="3"/>
+      <c r="C254" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="D254" s="3"/>
       <c r="E254" s="3" t="s">
         <v>6</v>
@@ -5942,7 +5980,9 @@
       <c r="B255" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C255" s="3"/>
+      <c r="C255" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="D255" s="3"/>
       <c r="E255" s="3" t="s">
         <v>6</v>
@@ -5962,7 +6002,9 @@
       <c r="B256" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C256" s="3"/>
+      <c r="C256" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="D256" s="3"/>
       <c r="E256" s="3" t="s">
         <v>6</v>
@@ -5982,7 +6024,9 @@
       <c r="B257" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C257" s="3"/>
+      <c r="C257" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="D257" s="3"/>
       <c r="E257" s="3" t="s">
         <v>6</v>
@@ -6002,7 +6046,9 @@
       <c r="B258" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C258" s="3"/>
+      <c r="C258" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="D258" s="3"/>
       <c r="E258" s="3" t="s">
         <v>6</v>
@@ -6022,7 +6068,9 @@
       <c r="B259" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C259" s="3"/>
+      <c r="C259" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="D259" s="3"/>
       <c r="E259" s="3" t="s">
         <v>6</v>
@@ -6042,7 +6090,9 @@
       <c r="B260" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C260" s="3"/>
+      <c r="C260" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="D260" s="3"/>
       <c r="E260" s="3" t="s">
         <v>6</v>
@@ -6062,7 +6112,9 @@
       <c r="B261" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C261" s="3"/>
+      <c r="C261" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="D261" s="3"/>
       <c r="E261" s="3" t="s">
         <v>6</v>
@@ -6082,7 +6134,9 @@
       <c r="B262" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C262" s="3"/>
+      <c r="C262" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="D262" s="3"/>
       <c r="E262" s="3" t="s">
         <v>6</v>
@@ -6102,7 +6156,9 @@
       <c r="B263" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C263" s="3"/>
+      <c r="C263" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="D263" s="3"/>
       <c r="E263" s="3" t="s">
         <v>6</v>
@@ -6122,7 +6178,9 @@
       <c r="B264" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C264" s="3"/>
+      <c r="C264" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="D264" s="3"/>
       <c r="E264" s="3" t="s">
         <v>6</v>
@@ -6142,7 +6200,9 @@
       <c r="B265" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C265" s="3"/>
+      <c r="C265" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="D265" s="3"/>
       <c r="E265" s="3" t="s">
         <v>6</v>
@@ -6162,7 +6222,9 @@
       <c r="B266" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C266" s="3"/>
+      <c r="C266" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="D266" s="3"/>
       <c r="E266" s="3" t="s">
         <v>6</v>
@@ -6182,7 +6244,9 @@
       <c r="B267" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C267" s="3"/>
+      <c r="C267" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="D267" s="3"/>
       <c r="E267" s="3" t="s">
         <v>6</v>
@@ -6202,7 +6266,9 @@
       <c r="B268" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C268" s="3"/>
+      <c r="C268" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="D268" s="3"/>
       <c r="E268" s="3" t="s">
         <v>6</v>
@@ -6222,7 +6288,9 @@
       <c r="B269" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C269" s="3"/>
+      <c r="C269" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="D269" s="3"/>
       <c r="E269" s="3" t="s">
         <v>6</v>
@@ -6242,7 +6310,9 @@
       <c r="B270" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C270" s="3"/>
+      <c r="C270" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="D270" s="3"/>
       <c r="E270" s="3" t="s">
         <v>6</v>
@@ -6262,7 +6332,9 @@
       <c r="B271" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C271" s="3"/>
+      <c r="C271" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="D271" s="3"/>
       <c r="E271" s="3" t="s">
         <v>6</v>
@@ -6282,7 +6354,9 @@
       <c r="B272" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C272" s="3"/>
+      <c r="C272" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="D272" s="3"/>
       <c r="E272" s="3" t="s">
         <v>6</v>
@@ -6302,7 +6376,9 @@
       <c r="B273" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C273" s="3"/>
+      <c r="C273" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="D273" s="3"/>
       <c r="E273" s="3" t="s">
         <v>6</v>
@@ -6322,7 +6398,9 @@
       <c r="B274" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C274" s="3"/>
+      <c r="C274" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="D274" s="3"/>
       <c r="E274" s="3" t="s">
         <v>6</v>
@@ -6342,7 +6420,9 @@
       <c r="B275" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C275" s="3"/>
+      <c r="C275" s="3" t="s">
+        <v>132</v>
+      </c>
       <c r="D275" s="3"/>
       <c r="E275" s="3" t="s">
         <v>6</v>
@@ -6362,7 +6442,9 @@
       <c r="B276" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C276" s="3"/>
+      <c r="C276" s="3" t="s">
+        <v>132</v>
+      </c>
       <c r="D276" s="3"/>
       <c r="E276" s="3" t="s">
         <v>6</v>
@@ -6382,7 +6464,9 @@
       <c r="B277" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C277" s="3"/>
+      <c r="C277" s="3" t="s">
+        <v>132</v>
+      </c>
       <c r="D277" s="3"/>
       <c r="E277" s="3" t="s">
         <v>6</v>
@@ -6402,7 +6486,9 @@
       <c r="B278" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C278" s="3"/>
+      <c r="C278" s="3" t="s">
+        <v>130</v>
+      </c>
       <c r="D278" s="3"/>
       <c r="E278" s="3" t="s">
         <v>6</v>
@@ -6422,7 +6508,9 @@
       <c r="B279" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C279" s="3"/>
+      <c r="C279" s="3" t="s">
+        <v>132</v>
+      </c>
       <c r="D279" s="3"/>
       <c r="E279" s="3" t="s">
         <v>6</v>
@@ -6442,7 +6530,9 @@
       <c r="B280" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C280" s="3"/>
+      <c r="C280" s="3" t="s">
+        <v>132</v>
+      </c>
       <c r="D280" s="3"/>
       <c r="E280" s="3" t="s">
         <v>6</v>
@@ -6462,7 +6552,9 @@
       <c r="B281" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C281" s="3"/>
+      <c r="C281" s="3" t="s">
+        <v>132</v>
+      </c>
       <c r="D281" s="3"/>
       <c r="E281" s="3" t="s">
         <v>6</v>
@@ -6482,7 +6574,9 @@
       <c r="B282" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C282" s="3"/>
+      <c r="C282" s="3" t="s">
+        <v>132</v>
+      </c>
       <c r="D282" s="3"/>
       <c r="E282" s="3" t="s">
         <v>6</v>
@@ -6502,7 +6596,9 @@
       <c r="B283" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C283" s="3"/>
+      <c r="C283" s="3" t="s">
+        <v>132</v>
+      </c>
       <c r="D283" s="3"/>
       <c r="E283" s="3" t="s">
         <v>6</v>
@@ -6522,7 +6618,9 @@
       <c r="B284" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C284" s="3"/>
+      <c r="C284" s="3" t="s">
+        <v>132</v>
+      </c>
       <c r="D284" s="3"/>
       <c r="E284" s="3" t="s">
         <v>6</v>
@@ -6542,7 +6640,9 @@
       <c r="B285" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C285" s="3"/>
+      <c r="C285" s="3" t="s">
+        <v>132</v>
+      </c>
       <c r="D285" s="3"/>
       <c r="E285" s="3" t="s">
         <v>6</v>
@@ -6562,7 +6662,9 @@
       <c r="B286" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C286" s="3"/>
+      <c r="C286" s="3" t="s">
+        <v>132</v>
+      </c>
       <c r="D286" s="3"/>
       <c r="E286" s="3" t="s">
         <v>6</v>
@@ -6582,7 +6684,9 @@
       <c r="B287" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C287" s="3"/>
+      <c r="C287" s="3" t="s">
+        <v>132</v>
+      </c>
       <c r="D287" s="3"/>
       <c r="E287" s="3" t="s">
         <v>6</v>
@@ -6602,7 +6706,9 @@
       <c r="B288" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C288" s="3"/>
+      <c r="C288" s="3" t="s">
+        <v>132</v>
+      </c>
       <c r="D288" s="3"/>
       <c r="E288" s="3" t="s">
         <v>6</v>
@@ -6622,7 +6728,9 @@
       <c r="B289" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C289" s="3"/>
+      <c r="C289" s="3" t="s">
+        <v>132</v>
+      </c>
       <c r="D289" s="3"/>
       <c r="E289" s="3" t="s">
         <v>6</v>
@@ -6642,7 +6750,9 @@
       <c r="B290" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C290" s="3"/>
+      <c r="C290" s="3" t="s">
+        <v>132</v>
+      </c>
       <c r="D290" s="3"/>
       <c r="E290" s="3" t="s">
         <v>6</v>
@@ -6662,7 +6772,9 @@
       <c r="B291" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C291" s="3"/>
+      <c r="C291" s="3" t="s">
+        <v>132</v>
+      </c>
       <c r="D291" s="3"/>
       <c r="E291" s="3" t="s">
         <v>6</v>
@@ -6682,7 +6794,9 @@
       <c r="B292" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C292" s="3"/>
+      <c r="C292" s="3" t="s">
+        <v>132</v>
+      </c>
       <c r="D292" s="3"/>
       <c r="E292" s="3" t="s">
         <v>6</v>
@@ -6702,7 +6816,9 @@
       <c r="B293" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C293" s="3"/>
+      <c r="C293" s="3" t="s">
+        <v>132</v>
+      </c>
       <c r="D293" s="3"/>
       <c r="E293" s="3" t="s">
         <v>6</v>
@@ -6722,7 +6838,9 @@
       <c r="B294" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C294" s="3"/>
+      <c r="C294" s="3" t="s">
+        <v>132</v>
+      </c>
       <c r="D294" s="3"/>
       <c r="E294" s="3" t="s">
         <v>6</v>
@@ -6742,7 +6860,9 @@
       <c r="B295" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C295" s="3"/>
+      <c r="C295" s="3" t="s">
+        <v>132</v>
+      </c>
       <c r="D295" s="3"/>
       <c r="E295" s="3" t="s">
         <v>6</v>
@@ -6762,7 +6882,9 @@
       <c r="B296" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C296" s="3"/>
+      <c r="C296" s="3" t="s">
+        <v>132</v>
+      </c>
       <c r="D296" s="3"/>
       <c r="E296" s="3" t="s">
         <v>6</v>
@@ -6802,7 +6924,9 @@
       <c r="B298" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="C298" s="3"/>
+      <c r="C298" s="3" t="s">
+        <v>129</v>
+      </c>
       <c r="D298" s="3"/>
       <c r="E298" s="3" t="s">
         <v>6</v>
@@ -14156,6 +14280,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>